<commit_message>
feat(equipment): bo sung dien thoai ban cho tat ca cac phong khu b va khu c
</commit_message>
<xml_diff>
--- a/danh_sach_thiet_bi_khu_A_moi.xlsx
+++ b/danh_sach_thiet_bi_khu_A_moi.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="226">
   <si>
     <t>Mã Serial</t>
   </si>
@@ -47,7 +47,7 @@
     <t>Treo tường đối diện giường ngủ</t>
   </si>
   <si>
-    <t>Trang bị mới Block A - Tầng 1</t>
+    <t>Trang bị Block A - Tầng 1</t>
   </si>
   <si>
     <t>BOX-A122</t>
@@ -59,9 +59,6 @@
     <t>Gắn sau Tivi / Kệ Tivi</t>
   </si>
   <si>
-    <t>Trang bị Block A - Tầng 1</t>
-  </si>
-  <si>
     <t>RMT-A122</t>
   </si>
   <si>
@@ -182,9 +179,6 @@
     <t>TV32-A222</t>
   </si>
   <si>
-    <t>Trang bị mới Block A - Tầng 2</t>
-  </si>
-  <si>
     <t>BOX-A222</t>
   </si>
   <si>
@@ -275,9 +269,6 @@
     <t>TV32-A322</t>
   </si>
   <si>
-    <t>Trang bị mới Block A - Tầng 3</t>
-  </si>
-  <si>
     <t>BOX-A322</t>
   </si>
   <si>
@@ -371,9 +362,6 @@
     <t>TV32-A422</t>
   </si>
   <si>
-    <t>Trang bị mới Block A - Tầng 4</t>
-  </si>
-  <si>
     <t>BOX-A422</t>
   </si>
   <si>
@@ -467,9 +455,6 @@
     <t>TV32-A522</t>
   </si>
   <si>
-    <t>Trang bị mới Block A - Tầng 5</t>
-  </si>
-  <si>
     <t>BOX-A522</t>
   </si>
   <si>
@@ -560,9 +545,6 @@
     <t>TV32-A622</t>
   </si>
   <si>
-    <t>Trang bị mới Block A - Tầng 6</t>
-  </si>
-  <si>
     <t>BOX-A622</t>
   </si>
   <si>
@@ -629,13 +611,10 @@
     <t>TV32-A721</t>
   </si>
   <si>
-    <t>Trang bị mới Block A - Tầng 7</t>
+    <t>Trang bị Block A - Tầng 7</t>
   </si>
   <si>
     <t>BOX-A721</t>
-  </si>
-  <si>
-    <t>Trang bị Block A - Tầng 7</t>
   </si>
   <si>
     <t>RMT-A721</t>
@@ -1158,15 +1137,15 @@
         <v>13</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>16</v>
       </c>
       <c r="C4" s="3">
         <v>122</v>
@@ -1175,18 +1154,18 @@
         <v>8</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>19</v>
       </c>
       <c r="C5" s="3">
         <v>122</v>
@@ -1195,18 +1174,18 @@
         <v>8</v>
       </c>
       <c r="E5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="C6" s="3">
         <v>122</v>
@@ -1215,15 +1194,15 @@
         <v>8</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>7</v>
@@ -1243,7 +1222,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>12</v>
@@ -1258,15 +1237,15 @@
         <v>13</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C9" s="3">
         <v>123</v>
@@ -1275,18 +1254,18 @@
         <v>8</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C10" s="3">
         <v>123</v>
@@ -1295,15 +1274,15 @@
         <v>8</v>
       </c>
       <c r="E10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>7</v>
@@ -1323,7 +1302,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>12</v>
@@ -1338,15 +1317,15 @@
         <v>13</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C13" s="3">
         <v>124</v>
@@ -1355,18 +1334,18 @@
         <v>8</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C14" s="3">
         <v>124</v>
@@ -1375,18 +1354,18 @@
         <v>8</v>
       </c>
       <c r="E14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C15" s="3">
         <v>124</v>
@@ -1395,15 +1374,15 @@
         <v>8</v>
       </c>
       <c r="E15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>7</v>
@@ -1423,7 +1402,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>12</v>
@@ -1438,15 +1417,15 @@
         <v>13</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C18" s="3">
         <v>125</v>
@@ -1455,18 +1434,18 @@
         <v>8</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C19" s="3">
         <v>125</v>
@@ -1475,15 +1454,15 @@
         <v>8</v>
       </c>
       <c r="E19" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>7</v>
@@ -1503,7 +1482,7 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>12</v>
@@ -1518,15 +1497,15 @@
         <v>13</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C22" s="3">
         <v>126</v>
@@ -1535,18 +1514,18 @@
         <v>8</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C23" s="3">
         <v>126</v>
@@ -1555,18 +1534,18 @@
         <v>8</v>
       </c>
       <c r="E23" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C24" s="3">
         <v>126</v>
@@ -1575,18 +1554,18 @@
         <v>8</v>
       </c>
       <c r="E24" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>45</v>
       </c>
       <c r="C25" s="3">
         <v>221</v>
@@ -1595,15 +1574,15 @@
         <v>8</v>
       </c>
       <c r="E25" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>12</v>
@@ -1618,15 +1597,15 @@
         <v>13</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C27" s="3">
         <v>221</v>
@@ -1635,18 +1614,18 @@
         <v>8</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C28" s="3">
         <v>221</v>
@@ -1655,18 +1634,18 @@
         <v>8</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C29" s="3">
         <v>221</v>
@@ -1675,15 +1654,15 @@
         <v>8</v>
       </c>
       <c r="E29" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F29" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>7</v>
@@ -1698,12 +1677,12 @@
         <v>9</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>12</v>
@@ -1718,15 +1697,15 @@
         <v>13</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C32" s="3">
         <v>222</v>
@@ -1735,18 +1714,18 @@
         <v>8</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C33" s="3">
         <v>222</v>
@@ -1755,18 +1734,18 @@
         <v>8</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C34" s="3">
         <v>223</v>
@@ -1775,15 +1754,15 @@
         <v>8</v>
       </c>
       <c r="E34" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>12</v>
@@ -1798,15 +1777,15 @@
         <v>13</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C36" s="3">
         <v>223</v>
@@ -1815,18 +1794,18 @@
         <v>8</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C37" s="3">
         <v>223</v>
@@ -1835,18 +1814,18 @@
         <v>8</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C38" s="3">
         <v>223</v>
@@ -1855,15 +1834,15 @@
         <v>8</v>
       </c>
       <c r="E38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F38" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>7</v>
@@ -1878,12 +1857,12 @@
         <v>9</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>12</v>
@@ -1898,15 +1877,15 @@
         <v>13</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C41" s="3">
         <v>224</v>
@@ -1915,18 +1894,18 @@
         <v>8</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42" spans="1:6">
       <c r="A42" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C42" s="3">
         <v>224</v>
@@ -1935,18 +1914,18 @@
         <v>8</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C43" s="3">
         <v>225</v>
@@ -1955,15 +1934,15 @@
         <v>8</v>
       </c>
       <c r="E43" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="44" spans="1:6">
       <c r="A44" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>12</v>
@@ -1978,15 +1957,15 @@
         <v>13</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45" spans="1:6">
       <c r="A45" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C45" s="3">
         <v>225</v>
@@ -1995,18 +1974,18 @@
         <v>8</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="46" spans="1:6">
       <c r="A46" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C46" s="3">
         <v>225</v>
@@ -2015,18 +1994,18 @@
         <v>8</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="47" spans="1:6">
       <c r="A47" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C47" s="3">
         <v>225</v>
@@ -2035,15 +2014,15 @@
         <v>8</v>
       </c>
       <c r="E47" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F47" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F47" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="48" spans="1:6">
       <c r="A48" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>7</v>
@@ -2058,12 +2037,12 @@
         <v>9</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="49" spans="1:6">
       <c r="A49" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>12</v>
@@ -2078,15 +2057,15 @@
         <v>13</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:6">
       <c r="A50" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C50" s="3">
         <v>226</v>
@@ -2095,18 +2074,18 @@
         <v>8</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:6">
       <c r="A51" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C51" s="3">
         <v>226</v>
@@ -2115,18 +2094,18 @@
         <v>8</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="52" spans="1:6">
       <c r="A52" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C52" s="3">
         <v>321</v>
@@ -2135,15 +2114,15 @@
         <v>8</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="53" spans="1:6">
       <c r="A53" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>12</v>
@@ -2158,15 +2137,15 @@
         <v>13</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="54" spans="1:6">
       <c r="A54" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C54" s="3">
         <v>321</v>
@@ -2175,18 +2154,18 @@
         <v>8</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="55" spans="1:6">
       <c r="A55" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C55" s="3">
         <v>321</v>
@@ -2195,18 +2174,18 @@
         <v>8</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C56" s="3">
         <v>321</v>
@@ -2215,15 +2194,15 @@
         <v>8</v>
       </c>
       <c r="E56" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F56" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="57" spans="1:6">
       <c r="A57" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>7</v>
@@ -2238,12 +2217,12 @@
         <v>9</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="3" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>12</v>
@@ -2258,15 +2237,15 @@
         <v>13</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C59" s="3">
         <v>322</v>
@@ -2275,18 +2254,18 @@
         <v>8</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="60" spans="1:6">
       <c r="A60" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C60" s="3">
         <v>322</v>
@@ -2295,35 +2274,35 @@
         <v>8</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="61" spans="1:6">
       <c r="A61" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C61" s="3">
         <v>323</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="62" spans="1:6">
       <c r="A62" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>12</v>
@@ -2338,15 +2317,15 @@
         <v>13</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="63" spans="1:6">
       <c r="A63" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C63" s="3">
         <v>323</v>
@@ -2355,18 +2334,18 @@
         <v>8</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="64" spans="1:6">
       <c r="A64" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C64" s="3">
         <v>323</v>
@@ -2375,18 +2354,18 @@
         <v>8</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="65" spans="1:6">
       <c r="A65" s="3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C65" s="3">
         <v>323</v>
@@ -2395,15 +2374,15 @@
         <v>8</v>
       </c>
       <c r="E65" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F65" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F65" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="66" spans="1:6">
       <c r="A66" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>7</v>
@@ -2418,12 +2397,12 @@
         <v>9</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
     </row>
     <row r="67" spans="1:6">
       <c r="A67" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>12</v>
@@ -2438,15 +2417,15 @@
         <v>13</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="68" spans="1:6">
       <c r="A68" s="3" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C68" s="3">
         <v>324</v>
@@ -2455,18 +2434,18 @@
         <v>8</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="69" spans="1:6">
       <c r="A69" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C69" s="3">
         <v>324</v>
@@ -2475,15 +2454,15 @@
         <v>8</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="70" spans="1:6">
       <c r="A70" s="3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>12</v>
@@ -2498,15 +2477,15 @@
         <v>13</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="71" spans="1:6">
       <c r="A71" s="3" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C71" s="3">
         <v>325</v>
@@ -2515,18 +2494,18 @@
         <v>8</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="72" spans="1:6">
       <c r="A72" s="3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C72" s="3">
         <v>325</v>
@@ -2535,18 +2514,18 @@
         <v>8</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="73" spans="1:6">
       <c r="A73" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C73" s="3">
         <v>325</v>
@@ -2555,15 +2534,15 @@
         <v>8</v>
       </c>
       <c r="E73" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F73" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="74" spans="1:6">
       <c r="A74" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>7</v>
@@ -2578,12 +2557,12 @@
         <v>9</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
     </row>
     <row r="75" spans="1:6">
       <c r="A75" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>12</v>
@@ -2598,15 +2577,15 @@
         <v>13</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="76" spans="1:6">
       <c r="A76" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C76" s="3">
         <v>326</v>
@@ -2615,18 +2594,18 @@
         <v>8</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="77" spans="1:6">
       <c r="A77" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C77" s="3">
         <v>326</v>
@@ -2635,35 +2614,35 @@
         <v>8</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="78" spans="1:6">
       <c r="A78" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C78" s="3">
         <v>421</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="79" spans="1:6">
       <c r="A79" s="3" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>12</v>
@@ -2678,15 +2657,15 @@
         <v>13</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="80" spans="1:6">
       <c r="A80" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C80" s="3">
         <v>421</v>
@@ -2695,18 +2674,18 @@
         <v>8</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="81" spans="1:6">
       <c r="A81" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C81" s="3">
         <v>421</v>
@@ -2715,18 +2694,18 @@
         <v>8</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="82" spans="1:6">
       <c r="A82" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C82" s="3">
         <v>421</v>
@@ -2735,15 +2714,15 @@
         <v>8</v>
       </c>
       <c r="E82" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F82" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F82" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="83" spans="1:6">
       <c r="A83" s="3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>7</v>
@@ -2758,12 +2737,12 @@
         <v>9</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
     </row>
     <row r="84" spans="1:6">
       <c r="A84" s="3" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>12</v>
@@ -2778,15 +2757,15 @@
         <v>13</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="85" spans="1:6">
       <c r="A85" s="3" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C85" s="3">
         <v>422</v>
@@ -2795,18 +2774,18 @@
         <v>8</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="86" spans="1:6">
       <c r="A86" s="3" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C86" s="3">
         <v>422</v>
@@ -2815,18 +2794,18 @@
         <v>8</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="87" spans="1:6">
       <c r="A87" s="3" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C87" s="3">
         <v>423</v>
@@ -2835,15 +2814,15 @@
         <v>8</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="88" spans="1:6">
       <c r="A88" s="3" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>12</v>
@@ -2858,15 +2837,15 @@
         <v>13</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="89" spans="1:6">
       <c r="A89" s="3" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C89" s="3">
         <v>423</v>
@@ -2875,18 +2854,18 @@
         <v>8</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="90" spans="1:6">
       <c r="A90" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C90" s="3">
         <v>423</v>
@@ -2895,18 +2874,18 @@
         <v>8</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="91" spans="1:6">
       <c r="A91" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C91" s="3">
         <v>423</v>
@@ -2915,15 +2894,15 @@
         <v>8</v>
       </c>
       <c r="E91" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F91" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F91" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="92" spans="1:6">
       <c r="A92" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>7</v>
@@ -2938,12 +2917,12 @@
         <v>9</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
     </row>
     <row r="93" spans="1:6">
       <c r="A93" s="3" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>12</v>
@@ -2958,15 +2937,15 @@
         <v>13</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="94" spans="1:6">
       <c r="A94" s="3" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C94" s="3">
         <v>424</v>
@@ -2975,18 +2954,18 @@
         <v>8</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="95" spans="1:6">
       <c r="A95" s="3" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C95" s="3">
         <v>424</v>
@@ -2995,18 +2974,18 @@
         <v>8</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="96" spans="1:6">
       <c r="A96" s="3" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C96" s="3">
         <v>425</v>
@@ -3015,15 +2994,15 @@
         <v>8</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="97" spans="1:6">
       <c r="A97" s="3" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>12</v>
@@ -3038,15 +3017,15 @@
         <v>13</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="98" spans="1:6">
       <c r="A98" s="3" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C98" s="3">
         <v>425</v>
@@ -3055,18 +3034,18 @@
         <v>8</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="99" spans="1:6">
       <c r="A99" s="3" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C99" s="3">
         <v>425</v>
@@ -3075,18 +3054,18 @@
         <v>8</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="100" spans="1:6">
       <c r="A100" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C100" s="3">
         <v>425</v>
@@ -3095,15 +3074,15 @@
         <v>8</v>
       </c>
       <c r="E100" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F100" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F100" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="101" spans="1:6">
       <c r="A101" s="3" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>7</v>
@@ -3118,12 +3097,12 @@
         <v>9</v>
       </c>
       <c r="F101" s="2" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
     </row>
     <row r="102" spans="1:6">
       <c r="A102" s="3" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>12</v>
@@ -3138,15 +3117,15 @@
         <v>13</v>
       </c>
       <c r="F102" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="103" spans="1:6">
       <c r="A103" s="3" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C103" s="3">
         <v>426</v>
@@ -3155,18 +3134,18 @@
         <v>8</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="104" spans="1:6">
       <c r="A104" s="3" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C104" s="3">
         <v>426</v>
@@ -3175,18 +3154,18 @@
         <v>8</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="105" spans="1:6">
       <c r="A105" s="3" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C105" s="3">
         <v>521</v>
@@ -3195,15 +3174,15 @@
         <v>8</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="106" spans="1:6">
       <c r="A106" s="3" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>12</v>
@@ -3218,15 +3197,15 @@
         <v>13</v>
       </c>
       <c r="F106" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="107" spans="1:6">
       <c r="A107" s="3" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C107" s="3">
         <v>521</v>
@@ -3235,18 +3214,18 @@
         <v>8</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F107" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="108" spans="1:6">
       <c r="A108" s="3" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C108" s="3">
         <v>521</v>
@@ -3255,18 +3234,18 @@
         <v>8</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="109" spans="1:6">
       <c r="A109" s="3" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C109" s="3">
         <v>521</v>
@@ -3275,15 +3254,15 @@
         <v>8</v>
       </c>
       <c r="E109" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F109" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F109" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="110" spans="1:6">
       <c r="A110" s="3" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>7</v>
@@ -3298,12 +3277,12 @@
         <v>9</v>
       </c>
       <c r="F110" s="2" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="111" spans="1:6">
       <c r="A111" s="3" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>12</v>
@@ -3318,15 +3297,15 @@
         <v>13</v>
       </c>
       <c r="F111" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="112" spans="1:6">
       <c r="A112" s="3" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C112" s="3">
         <v>522</v>
@@ -3335,18 +3314,18 @@
         <v>8</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F112" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="113" spans="1:6">
       <c r="A113" s="3" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C113" s="3">
         <v>522</v>
@@ -3355,18 +3334,18 @@
         <v>8</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="114" spans="1:6">
       <c r="A114" s="3" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C114" s="3">
         <v>523</v>
@@ -3375,15 +3354,15 @@
         <v>8</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F114" s="2" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="115" spans="1:6">
       <c r="A115" s="3" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>12</v>
@@ -3398,15 +3377,15 @@
         <v>13</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="116" spans="1:6">
       <c r="A116" s="3" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C116" s="3">
         <v>523</v>
@@ -3415,18 +3394,18 @@
         <v>8</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F116" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="117" spans="1:6">
       <c r="A117" s="3" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C117" s="3">
         <v>523</v>
@@ -3435,18 +3414,18 @@
         <v>8</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F117" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="118" spans="1:6">
       <c r="A118" s="3" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C118" s="3">
         <v>523</v>
@@ -3455,15 +3434,15 @@
         <v>8</v>
       </c>
       <c r="E118" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F118" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F118" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="119" spans="1:6">
       <c r="A119" s="3" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="B119" s="2" t="s">
         <v>7</v>
@@ -3478,12 +3457,12 @@
         <v>9</v>
       </c>
       <c r="F119" s="2" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="120" spans="1:6">
       <c r="A120" s="3" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>12</v>
@@ -3498,15 +3477,15 @@
         <v>13</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="121" spans="1:6">
       <c r="A121" s="3" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C121" s="3">
         <v>524</v>
@@ -3515,18 +3494,18 @@
         <v>8</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="122" spans="1:6">
       <c r="A122" s="3" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C122" s="3">
         <v>524</v>
@@ -3535,18 +3514,18 @@
         <v>8</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="123" spans="1:6">
       <c r="A123" s="3" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C123" s="3">
         <v>525</v>
@@ -3555,15 +3534,15 @@
         <v>8</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="124" spans="1:6">
       <c r="A124" s="3" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>12</v>
@@ -3578,15 +3557,15 @@
         <v>13</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="125" spans="1:6">
       <c r="A125" s="3" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C125" s="3">
         <v>525</v>
@@ -3595,18 +3574,18 @@
         <v>8</v>
       </c>
       <c r="E125" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F125" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="126" spans="1:6">
       <c r="A126" s="3" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C126" s="3">
         <v>525</v>
@@ -3615,18 +3594,18 @@
         <v>8</v>
       </c>
       <c r="E126" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F126" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="127" spans="1:6">
       <c r="A127" s="3" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C127" s="3">
         <v>525</v>
@@ -3635,15 +3614,15 @@
         <v>8</v>
       </c>
       <c r="E127" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F127" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F127" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="128" spans="1:6">
       <c r="A128" s="3" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>7</v>
@@ -3658,12 +3637,12 @@
         <v>9</v>
       </c>
       <c r="F128" s="2" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="129" spans="1:6">
       <c r="A129" s="3" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>12</v>
@@ -3678,15 +3657,15 @@
         <v>13</v>
       </c>
       <c r="F129" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="130" spans="1:6">
       <c r="A130" s="3" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C130" s="3">
         <v>526</v>
@@ -3695,18 +3674,18 @@
         <v>8</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F130" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="131" spans="1:6">
       <c r="A131" s="3" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C131" s="3">
         <v>526</v>
@@ -3715,18 +3694,18 @@
         <v>8</v>
       </c>
       <c r="E131" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F131" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="132" spans="1:6">
       <c r="A132" s="3" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C132" s="3">
         <v>621</v>
@@ -3735,15 +3714,15 @@
         <v>8</v>
       </c>
       <c r="E132" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F132" s="2" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
     </row>
     <row r="133" spans="1:6">
       <c r="A133" s="3" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="B133" s="2" t="s">
         <v>12</v>
@@ -3758,15 +3737,15 @@
         <v>13</v>
       </c>
       <c r="F133" s="2" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="134" spans="1:6">
       <c r="A134" s="3" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C134" s="3">
         <v>621</v>
@@ -3775,18 +3754,18 @@
         <v>8</v>
       </c>
       <c r="E134" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F134" s="2" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="135" spans="1:6">
       <c r="A135" s="3" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C135" s="3">
         <v>621</v>
@@ -3795,18 +3774,18 @@
         <v>8</v>
       </c>
       <c r="E135" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F135" s="2" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="136" spans="1:6">
       <c r="A136" s="3" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C136" s="3">
         <v>621</v>
@@ -3815,15 +3794,15 @@
         <v>8</v>
       </c>
       <c r="E136" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F136" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F136" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="137" spans="1:6">
       <c r="A137" s="3" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="B137" s="2" t="s">
         <v>7</v>
@@ -3838,12 +3817,12 @@
         <v>9</v>
       </c>
       <c r="F137" s="2" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
     </row>
     <row r="138" spans="1:6">
       <c r="A138" s="3" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="B138" s="2" t="s">
         <v>12</v>
@@ -3858,15 +3837,15 @@
         <v>13</v>
       </c>
       <c r="F138" s="2" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="139" spans="1:6">
       <c r="A139" s="3" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C139" s="3">
         <v>622</v>
@@ -3875,18 +3854,18 @@
         <v>8</v>
       </c>
       <c r="E139" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F139" s="2" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="140" spans="1:6">
       <c r="A140" s="3" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C140" s="3">
         <v>622</v>
@@ -3895,18 +3874,18 @@
         <v>8</v>
       </c>
       <c r="E140" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F140" s="2" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="141" spans="1:6">
       <c r="A141" s="3" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C141" s="3">
         <v>623</v>
@@ -3915,15 +3894,15 @@
         <v>8</v>
       </c>
       <c r="E141" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F141" s="2" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
     </row>
     <row r="142" spans="1:6">
       <c r="A142" s="3" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="B142" s="2" t="s">
         <v>12</v>
@@ -3938,15 +3917,15 @@
         <v>13</v>
       </c>
       <c r="F142" s="2" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="143" spans="1:6">
       <c r="A143" s="3" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C143" s="3">
         <v>623</v>
@@ -3955,18 +3934,18 @@
         <v>8</v>
       </c>
       <c r="E143" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F143" s="2" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="144" spans="1:6">
       <c r="A144" s="3" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C144" s="3">
         <v>623</v>
@@ -3975,18 +3954,18 @@
         <v>8</v>
       </c>
       <c r="E144" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F144" s="2" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="145" spans="1:6">
       <c r="A145" s="3" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C145" s="3">
         <v>623</v>
@@ -3995,15 +3974,15 @@
         <v>8</v>
       </c>
       <c r="E145" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F145" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F145" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="146" spans="1:6">
       <c r="A146" s="3" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="B146" s="2" t="s">
         <v>7</v>
@@ -4018,12 +3997,12 @@
         <v>9</v>
       </c>
       <c r="F146" s="2" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
     </row>
     <row r="147" spans="1:6">
       <c r="A147" s="3" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="B147" s="2" t="s">
         <v>12</v>
@@ -4038,15 +4017,15 @@
         <v>13</v>
       </c>
       <c r="F147" s="2" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="148" spans="1:6">
       <c r="A148" s="3" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C148" s="3">
         <v>624</v>
@@ -4055,18 +4034,18 @@
         <v>8</v>
       </c>
       <c r="E148" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F148" s="2" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="149" spans="1:6">
       <c r="A149" s="3" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C149" s="3">
         <v>624</v>
@@ -4075,18 +4054,18 @@
         <v>8</v>
       </c>
       <c r="E149" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F149" s="2" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="150" spans="1:6">
       <c r="A150" s="3" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C150" s="3">
         <v>625</v>
@@ -4095,15 +4074,15 @@
         <v>8</v>
       </c>
       <c r="E150" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F150" s="2" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
     </row>
     <row r="151" spans="1:6">
       <c r="A151" s="3" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="B151" s="2" t="s">
         <v>12</v>
@@ -4118,15 +4097,15 @@
         <v>13</v>
       </c>
       <c r="F151" s="2" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="152" spans="1:6">
       <c r="A152" s="3" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C152" s="3">
         <v>625</v>
@@ -4135,18 +4114,18 @@
         <v>8</v>
       </c>
       <c r="E152" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F152" s="2" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="153" spans="1:6">
       <c r="A153" s="3" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C153" s="3">
         <v>625</v>
@@ -4155,18 +4134,18 @@
         <v>8</v>
       </c>
       <c r="E153" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F153" s="2" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="154" spans="1:6">
       <c r="A154" s="3" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C154" s="3">
         <v>625</v>
@@ -4175,15 +4154,15 @@
         <v>8</v>
       </c>
       <c r="E154" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F154" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F154" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="155" spans="1:6">
       <c r="A155" s="3" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="B155" s="2" t="s">
         <v>7</v>
@@ -4198,12 +4177,12 @@
         <v>9</v>
       </c>
       <c r="F155" s="2" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
     </row>
     <row r="156" spans="1:6">
       <c r="A156" s="3" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="B156" s="2" t="s">
         <v>12</v>
@@ -4218,15 +4197,15 @@
         <v>13</v>
       </c>
       <c r="F156" s="2" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="157" spans="1:6">
       <c r="A157" s="3" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C157" s="3">
         <v>626</v>
@@ -4235,18 +4214,18 @@
         <v>8</v>
       </c>
       <c r="E157" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F157" s="2" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="158" spans="1:6">
       <c r="A158" s="3" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C158" s="3">
         <v>626</v>
@@ -4255,15 +4234,15 @@
         <v>8</v>
       </c>
       <c r="E158" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F158" s="2" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="159" spans="1:6">
       <c r="A159" s="3" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="B159" s="2" t="s">
         <v>7</v>
@@ -4278,12 +4257,12 @@
         <v>9</v>
       </c>
       <c r="F159" s="2" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
     </row>
     <row r="160" spans="1:6">
       <c r="A160" s="3" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="B160" s="2" t="s">
         <v>12</v>
@@ -4298,15 +4277,15 @@
         <v>13</v>
       </c>
       <c r="F160" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
     </row>
     <row r="161" spans="1:6">
       <c r="A161" s="3" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C161" s="3">
         <v>721</v>
@@ -4315,18 +4294,18 @@
         <v>8</v>
       </c>
       <c r="E161" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F161" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
     </row>
     <row r="162" spans="1:6">
       <c r="A162" s="3" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C162" s="3">
         <v>721</v>
@@ -4335,18 +4314,18 @@
         <v>8</v>
       </c>
       <c r="E162" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F162" s="2" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="163" spans="1:6">
       <c r="A163" s="3" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C163" s="3">
         <v>721</v>
@@ -4355,15 +4334,15 @@
         <v>8</v>
       </c>
       <c r="E163" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F163" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F163" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="164" spans="1:6">
       <c r="A164" s="3" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="B164" s="2" t="s">
         <v>7</v>
@@ -4378,12 +4357,12 @@
         <v>9</v>
       </c>
       <c r="F164" s="2" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
     </row>
     <row r="165" spans="1:6">
       <c r="A165" s="3" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="B165" s="2" t="s">
         <v>12</v>
@@ -4398,15 +4377,15 @@
         <v>13</v>
       </c>
       <c r="F165" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
     </row>
     <row r="166" spans="1:6">
       <c r="A166" s="3" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C166" s="3">
         <v>722</v>
@@ -4415,18 +4394,18 @@
         <v>8</v>
       </c>
       <c r="E166" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F166" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
     </row>
     <row r="167" spans="1:6">
       <c r="A167" s="3" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C167" s="3">
         <v>722</v>
@@ -4435,15 +4414,15 @@
         <v>8</v>
       </c>
       <c r="E167" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F167" s="2" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="168" spans="1:6">
       <c r="A168" s="3" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="B168" s="2" t="s">
         <v>7</v>
@@ -4458,12 +4437,12 @@
         <v>9</v>
       </c>
       <c r="F168" s="2" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
     </row>
     <row r="169" spans="1:6">
       <c r="A169" s="3" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="B169" s="2" t="s">
         <v>12</v>
@@ -4478,15 +4457,15 @@
         <v>13</v>
       </c>
       <c r="F169" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
     </row>
     <row r="170" spans="1:6">
       <c r="A170" s="3" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C170" s="3">
         <v>723</v>
@@ -4495,18 +4474,18 @@
         <v>8</v>
       </c>
       <c r="E170" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F170" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
     </row>
     <row r="171" spans="1:6">
       <c r="A171" s="3" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C171" s="3">
         <v>723</v>
@@ -4515,18 +4494,18 @@
         <v>8</v>
       </c>
       <c r="E171" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F171" s="2" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="172" spans="1:6">
       <c r="A172" s="3" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C172" s="3">
         <v>723</v>
@@ -4535,15 +4514,15 @@
         <v>8</v>
       </c>
       <c r="E172" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F172" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F172" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="173" spans="1:6">
       <c r="A173" s="3" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="B173" s="2" t="s">
         <v>7</v>
@@ -4558,12 +4537,12 @@
         <v>9</v>
       </c>
       <c r="F173" s="2" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
     </row>
     <row r="174" spans="1:6">
       <c r="A174" s="3" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="B174" s="2" t="s">
         <v>12</v>
@@ -4578,15 +4557,15 @@
         <v>13</v>
       </c>
       <c r="F174" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
     </row>
     <row r="175" spans="1:6">
       <c r="A175" s="3" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C175" s="3">
         <v>724</v>
@@ -4595,18 +4574,18 @@
         <v>8</v>
       </c>
       <c r="E175" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F175" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
     </row>
     <row r="176" spans="1:6">
       <c r="A176" s="3" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C176" s="3">
         <v>724</v>
@@ -4615,15 +4594,15 @@
         <v>8</v>
       </c>
       <c r="E176" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F176" s="2" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="177" spans="1:6">
       <c r="A177" s="3" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="B177" s="2" t="s">
         <v>7</v>
@@ -4638,12 +4617,12 @@
         <v>9</v>
       </c>
       <c r="F177" s="2" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
     </row>
     <row r="178" spans="1:6">
       <c r="A178" s="3" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="B178" s="2" t="s">
         <v>12</v>
@@ -4658,15 +4637,15 @@
         <v>13</v>
       </c>
       <c r="F178" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
     </row>
     <row r="179" spans="1:6">
       <c r="A179" s="3" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C179" s="3">
         <v>725</v>
@@ -4675,18 +4654,18 @@
         <v>8</v>
       </c>
       <c r="E179" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F179" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
     </row>
     <row r="180" spans="1:6">
       <c r="A180" s="3" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C180" s="3">
         <v>725</v>
@@ -4695,18 +4674,18 @@
         <v>8</v>
       </c>
       <c r="E180" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F180" s="2" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="181" spans="1:6">
       <c r="A181" s="3" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C181" s="3">
         <v>725</v>
@@ -4715,15 +4694,15 @@
         <v>8</v>
       </c>
       <c r="E181" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F181" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F181" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="182" spans="1:6">
       <c r="A182" s="3" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B182" s="2" t="s">
         <v>7</v>
@@ -4738,12 +4717,12 @@
         <v>9</v>
       </c>
       <c r="F182" s="2" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
     </row>
     <row r="183" spans="1:6">
       <c r="A183" s="3" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B183" s="2" t="s">
         <v>12</v>
@@ -4758,15 +4737,15 @@
         <v>13</v>
       </c>
       <c r="F183" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
     </row>
     <row r="184" spans="1:6">
       <c r="A184" s="3" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C184" s="3">
         <v>726</v>
@@ -4775,18 +4754,18 @@
         <v>8</v>
       </c>
       <c r="E184" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F184" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
     </row>
     <row r="185" spans="1:6">
       <c r="A185" s="3" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C185" s="3">
         <v>726</v>
@@ -4795,10 +4774,10 @@
         <v>8</v>
       </c>
       <c r="E185" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F185" s="2" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>